<commit_message>
Update Attendance Roster_Splunk Basics_VILT10400.xlsx
</commit_message>
<xml_diff>
--- a/Attendance Roster_Splunk Basics_VILT10400.xlsx
+++ b/Attendance Roster_Splunk Basics_VILT10400.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cisco-my.sharepoint.com/personal/davipaul_cisco_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\cisco_emea_05_03_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8507532E-0BA0-4429-9F03-0ED2E585EA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34ADCCDA-7201-4892-913C-F0A1080EF735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A2522E59-55AA-40D7-AE73-25FE8E1DAF04}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A2522E59-55AA-40D7-AE73-25FE8E1DAF04}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="46">
   <si>
     <t>Start Date</t>
   </si>
@@ -132,13 +131,55 @@
   </si>
   <si>
     <t>seethar</t>
+  </si>
+  <si>
+    <t>https://cloud.cdp.rpsconsulting.in/</t>
+  </si>
+  <si>
+    <t>25MMS5314_U01</t>
+  </si>
+  <si>
+    <t>P@%%w0rd@123</t>
+  </si>
+  <si>
+    <t>25MMS5314_U02</t>
+  </si>
+  <si>
+    <t>25MMS5314_U03</t>
+  </si>
+  <si>
+    <t>25MMS5314_U04</t>
+  </si>
+  <si>
+    <t>25MMS5314_U05</t>
+  </si>
+  <si>
+    <t>25MMS5314_U06</t>
+  </si>
+  <si>
+    <t>25MMS5314_U07</t>
+  </si>
+  <si>
+    <t>25MMS5314_U08</t>
+  </si>
+  <si>
+    <t>25MMS5314_U09</t>
+  </si>
+  <si>
+    <t>25MMS5314_U10</t>
+  </si>
+  <si>
+    <t>25MMS5314_U11</t>
+  </si>
+  <si>
+    <t>25MMS5314_U12</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -184,6 +225,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -369,18 +418,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -421,8 +465,19 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -756,224 +811,224 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F52638C-DE0B-4F65-821B-D3C54A2C1DB4}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="9.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-    </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="4">
         <v>46086</v>
       </c>
-      <c r="D3" s="7"/>
-    </row>
-    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="4"/>
-      <c r="B4" s="8" t="s">
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2"/>
+      <c r="B4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="7">
         <v>46087</v>
       </c>
-      <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="8" t="s">
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="8">
         <v>12</v>
       </c>
-      <c r="D5" s="7"/>
-    </row>
-    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4"/>
-      <c r="B6" s="11" t="s">
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="4"/>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="4"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
       <c r="B10" s="1"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="13">
         <v>46086</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="13">
         <v>46087</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="16" t="s">
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="16" t="s">
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="16" t="s">
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="16" t="s">
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="16" t="s">
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="18" t="s">
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="16" t="s">
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="18" t="s">
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="16" t="s">
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="16" t="s">
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -986,6 +1041,184 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{543A744B-4773-4489-B9EA-86AF7FD6273C}">
+  <dimension ref="B3:F19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C3" s="20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B8" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="17"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B9" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="17"/>
+    </row>
+    <row r="10" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B10" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="17"/>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="17"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="17"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="17"/>
+    </row>
+    <row r="14" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="17"/>
+    </row>
+    <row r="15" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" s="17"/>
+    </row>
+    <row r="16" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F16" s="17"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" s="17"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="17"/>
+    </row>
+    <row r="19" spans="2:6" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" s="17"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{DF95D759-43AE-4664-BB03-49EBE526D71A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{c8f49a32-fde3-48a5-9266-b5b0972a22dc}" enabled="1" method="Standard" siteId="{5ae1af62-9505-4097-a69a-c1553ef7840e}" contentBits="2" removed="0"/>

</xml_diff>